<commit_message>
moved the reset button on the 18650 version of the board so i needed to re-upload all of the files to GitHub
</commit_message>
<xml_diff>
--- a/PCB/18650/Fabrication/PickAndPlace_PCB_18650.xlsx
+++ b/PCB/18650/Fabrication/PickAndPlace_PCB_18650.xlsx
@@ -364,13 +364,13 @@
     <t>SW-SMD_L3.9-W3.0-P4.45</t>
   </si>
   <si>
-    <t>3.429mm</t>
-  </si>
-  <si>
-    <t>-6.223mm</t>
-  </si>
-  <si>
-    <t>5.614mm</t>
+    <t>12.345mm</t>
+  </si>
+  <si>
+    <t>-9.424mm</t>
+  </si>
+  <si>
+    <t>-7.239mm</t>
   </si>
   <si>
     <t>SW2</t>
@@ -2022,10 +2022,10 @@
         <v>118</v>
       </c>
       <c r="H18" t="s">
+        <v>117</v>
+      </c>
+      <c r="I18" t="s">
         <v>119</v>
-      </c>
-      <c r="I18" t="s">
-        <v>118</v>
       </c>
       <c r="J18">
         <v>2</v>
@@ -2034,7 +2034,7 @@
         <v>21</v>
       </c>
       <c r="L18">
-        <v>180</v>
+        <v>270</v>
       </c>
       <c r="M18" t="s">
         <v>22</v>

</xml_diff>